<commit_message>
follow-ups: Telegram Why button proven end to end through polling (no webhook); enquiry report Do this next from data only - overdue call-backs, uncalled enquiries, most common reason for no; invented offline-kit suggestion removed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sample-reports/enquiries-follow-up.xlsx
+++ b/docs/sample-reports/enquiries-follow-up.xlsx
@@ -136,7 +136,7 @@
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 call-back is due today.</t>
+          <t xml:space="preserve">1 call-back is overdue.</t>
         </is>
       </c>
     </row>
@@ -148,7 +148,7 @@
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 enquiry is older than 2 working days with no call - the form promised one by now.</t>
+          <t xml:space="preserve">1 enquiry has not been called yet; 1 of them is past the 2 working days the form promises.</t>
         </is>
       </c>
     </row>
@@ -160,93 +160,81 @@
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">1 enquiry has had no answer 3 times: try a different time of day, or close it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">•</t>
-        </is>
-      </c>
-      <c r="B8" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">The top reason for "no" is no reliable internet or WiFi (1 of 2): consider the offline kit option.</t>
+          <t xml:space="preserve">Most common reason for "no": No reliable internet or WiFi - 1 of 2 (50%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How it went</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">How it went</t>
-        </is>
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Enquiries received</t>
+        </is>
+      </c>
+      <c r="B10" s="0">
+        <v>6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Enquiries received</t>
+          <t xml:space="preserve">Called</t>
         </is>
       </c>
       <c r="B11" s="0">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Called</t>
+          <t xml:space="preserve">Became farmers</t>
         </is>
       </c>
       <c r="B12" s="0">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Became farmers</t>
-        </is>
-      </c>
-      <c r="B13" s="0">
-        <v>1</v>
+          <t xml:space="preserve">Conversion rate (%)</t>
+        </is>
+      </c>
+      <c r="B13" s="6">
+        <v>16.7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Conversion rate (%)</t>
+          <t xml:space="preserve">Average hours to first call</t>
         </is>
       </c>
       <c r="B14" s="6">
-        <v>16.7</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="0" t="inlineStr">
         <is>
-          <t xml:space="preserve">Average hours to first call</t>
-        </is>
-      </c>
-      <c r="B15" s="6">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Call-backs due</t>
-        </is>
-      </c>
-      <c r="B16" s="0">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Counts are for enquiries received in the period. Call-backs due and enquiries waiting are as of today.</t>
+          <t xml:space="preserve">Call-backs overdue</t>
+        </is>
+      </c>
+      <c r="B15" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Counts are for enquiries received in the period. Overdue call-backs and uncalled enquiries are as of when the report was made.</t>
         </is>
       </c>
     </row>

</xml_diff>